<commit_message>
chore: refresh Angola trade profile notebooks and reports
</commit_message>
<xml_diff>
--- a/reports/Angola_2.1.1_top_export_partners_reverse.xlsx
+++ b/reports/Angola_2.1.1_top_export_partners_reverse.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9481" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9437" uniqueCount="190">
   <si>
     <t>refYear</t>
   </si>
@@ -941,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2369"/>
+  <dimension ref="A1:J2358"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -76397,358 +76397,6 @@
         <v>38018109936.056</v>
       </c>
     </row>
-    <row r="2359" spans="1:10">
-      <c r="A2359" s="1">
-        <v>2360</v>
-      </c>
-      <c r="B2359">
-        <v>2025</v>
-      </c>
-      <c r="C2359" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2359" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2359">
-        <v>1</v>
-      </c>
-      <c r="F2359" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2359" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2359">
-        <v>1946222800.48</v>
-      </c>
-      <c r="I2359">
-        <v>0.582434070081104</v>
-      </c>
-      <c r="J2359">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2360" spans="1:10">
-      <c r="A2360" s="1">
-        <v>2367</v>
-      </c>
-      <c r="B2360">
-        <v>2025</v>
-      </c>
-      <c r="C2360" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2360" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2360">
-        <v>2</v>
-      </c>
-      <c r="F2360" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2360" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2360">
-        <v>928208659.2589999</v>
-      </c>
-      <c r="I2360">
-        <v>0.277779269240608</v>
-      </c>
-      <c r="J2360">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2361" spans="1:10">
-      <c r="A2361" s="1">
-        <v>2357</v>
-      </c>
-      <c r="B2361">
-        <v>2025</v>
-      </c>
-      <c r="C2361" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2361" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2361">
-        <v>3</v>
-      </c>
-      <c r="F2361" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2361" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2361">
-        <v>460118607</v>
-      </c>
-      <c r="I2361">
-        <v>0.1376968520402513</v>
-      </c>
-      <c r="J2361">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2362" spans="1:10">
-      <c r="A2362" s="1">
-        <v>2365</v>
-      </c>
-      <c r="B2362">
-        <v>2025</v>
-      </c>
-      <c r="C2362" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2362" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2362">
-        <v>4</v>
-      </c>
-      <c r="F2362" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2362" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2362">
-        <v>5712596.995</v>
-      </c>
-      <c r="I2362">
-        <v>0.001709573599543865</v>
-      </c>
-      <c r="J2362">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2363" spans="1:10">
-      <c r="A2363" s="1">
-        <v>2361</v>
-      </c>
-      <c r="B2363">
-        <v>2025</v>
-      </c>
-      <c r="C2363" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2363" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2363">
-        <v>5</v>
-      </c>
-      <c r="F2363" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2363" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2363">
-        <v>1055260.755</v>
-      </c>
-      <c r="I2363">
-        <v>0.0003158013647666259</v>
-      </c>
-      <c r="J2363">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2364" spans="1:10">
-      <c r="A2364" s="1">
-        <v>2359</v>
-      </c>
-      <c r="B2364">
-        <v>2025</v>
-      </c>
-      <c r="C2364" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2364" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2364">
-        <v>6</v>
-      </c>
-      <c r="F2364" t="s">
-        <v>74</v>
-      </c>
-      <c r="G2364" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2364">
-        <v>89611.382</v>
-      </c>
-      <c r="I2364">
-        <v>2.681744450377429E-05</v>
-      </c>
-      <c r="J2364">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2365" spans="1:10">
-      <c r="A2365" s="1">
-        <v>2363</v>
-      </c>
-      <c r="B2365">
-        <v>2025</v>
-      </c>
-      <c r="C2365" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2365" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2365">
-        <v>7</v>
-      </c>
-      <c r="F2365" t="s">
-        <v>156</v>
-      </c>
-      <c r="G2365" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2365">
-        <v>88800</v>
-      </c>
-      <c r="I2365">
-        <v>2.657462722687568E-05</v>
-      </c>
-      <c r="J2365">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2366" spans="1:10">
-      <c r="A2366" s="1">
-        <v>2358</v>
-      </c>
-      <c r="B2366">
-        <v>2025</v>
-      </c>
-      <c r="C2366" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2366" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2366">
-        <v>8</v>
-      </c>
-      <c r="F2366" t="s">
-        <v>166</v>
-      </c>
-      <c r="G2366" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2366">
-        <v>34869.484</v>
-      </c>
-      <c r="I2366">
-        <v>1.043517498753948E-05</v>
-      </c>
-      <c r="J2366">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2367" spans="1:10">
-      <c r="A2367" s="1">
-        <v>2362</v>
-      </c>
-      <c r="B2367">
-        <v>2025</v>
-      </c>
-      <c r="C2367" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2367" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2367">
-        <v>9</v>
-      </c>
-      <c r="F2367" t="s">
-        <v>141</v>
-      </c>
-      <c r="G2367" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2367">
-        <v>948.4059999999999</v>
-      </c>
-      <c r="I2367">
-        <v>2.838236025870749E-07</v>
-      </c>
-      <c r="J2367">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2368" spans="1:10">
-      <c r="A2368" s="1">
-        <v>2364</v>
-      </c>
-      <c r="B2368">
-        <v>2025</v>
-      </c>
-      <c r="C2368" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2368" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2368">
-        <v>10</v>
-      </c>
-      <c r="F2368" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2368" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2368">
-        <v>596</v>
-      </c>
-      <c r="I2368">
-        <v>1.783612367929944E-07</v>
-      </c>
-      <c r="J2368">
-        <v>3341533231.751</v>
-      </c>
-    </row>
-    <row r="2369" spans="1:10">
-      <c r="A2369" s="1">
-        <v>2366</v>
-      </c>
-      <c r="B2369">
-        <v>2025</v>
-      </c>
-      <c r="C2369" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2369" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2369">
-        <v>11</v>
-      </c>
-      <c r="F2369" t="s">
-        <v>169</v>
-      </c>
-      <c r="G2369" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2369">
-        <v>481.99</v>
-      </c>
-      <c r="I2369">
-        <v>1.442421686608312E-07</v>
-      </c>
-      <c r="J2369">
-        <v>3341533231.751</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>